<commit_message>
moved files for convenience
</commit_message>
<xml_diff>
--- a/docs/MOJO_FPGA_pinout.xlsx
+++ b/docs/MOJO_FPGA_pinout.xlsx
@@ -4375,40 +4375,40 @@
         <v>238</v>
       </c>
       <c r="B2" s="10">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>189</v>
+        <v>153</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>190</v>
-      </c>
-      <c r="E2" s="1">
-        <v>10</v>
-      </c>
-      <c r="F2" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E2" s="13">
+        <v>1</v>
+      </c>
+      <c r="F2" s="13" t="s">
         <v>279</v>
       </c>
-      <c r="G2" s="1">
-        <v>0</v>
-      </c>
-      <c r="H2" s="1" t="str">
+      <c r="G2" s="13">
+        <v>15</v>
+      </c>
+      <c r="H2" s="13" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F2,"&lt;",G2,"&gt;"" LOC = ",$C2," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;0&gt;" LOC = P8 | IOSTANDARD = LVCMOS33;</v>
-      </c>
-      <c r="I2" s="1">
-        <v>0</v>
-      </c>
-      <c r="J2" s="1" t="str">
-        <f xml:space="preserve"> CONCATENATE("NET """,$F2,"&lt;",I2,"&gt;"" LOC = ",$C2," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;0&gt;" LOC = P8 | IOSTANDARD = LVCMOS33;</v>
-      </c>
-      <c r="K2" s="1">
-        <v>0</v>
-      </c>
-      <c r="L2" s="1" t="str">
+        <v>NET "A&lt;15&gt;" LOC = P33 | IOSTANDARD = LVCMOS33;</v>
+      </c>
+      <c r="I2" s="13" t="s">
+        <v>300</v>
+      </c>
+      <c r="J2" s="13" t="str">
+        <f xml:space="preserve"> CONCATENATE("NET """,I2,""" LOC = ",$C2," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "VPP" LOC = P33 | IOSTANDARD = LVCMOS33;</v>
+      </c>
+      <c r="K2" s="13">
+        <v>14</v>
+      </c>
+      <c r="L2" s="13" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F2,"&lt;",K2,"&gt;"" LOC = ",$C2," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;0&gt;" LOC = P8 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;14&gt;" LOC = P33 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -4416,40 +4416,40 @@
         <v>238</v>
       </c>
       <c r="B3" s="10">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>185</v>
+        <v>157</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>186</v>
+        <v>158</v>
       </c>
       <c r="E3" s="1">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>279</v>
       </c>
       <c r="G3" s="1">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H3" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F3,"&lt;",G3,"&gt;"" LOC = ",$C3," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;1&gt;" LOC = P10 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;12&gt;" LOC = P30 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I3" s="1">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="J3" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F3,"&lt;",I3,"&gt;"" LOC = ",$C3," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;1&gt;" LOC = P10 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;12&gt;" LOC = P30 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K3" s="1">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L3" s="1" t="str">
-        <f t="shared" ref="L3:L15" si="0" xml:space="preserve"> CONCATENATE("NET """,$F3,"&lt;",K3,"&gt;"" LOC = ",$C3," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;1&gt;" LOC = P10 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F3,"&lt;",K3,"&gt;"" LOC = ",$C3," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;12&gt;" LOC = P30 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -4457,40 +4457,40 @@
         <v>238</v>
       </c>
       <c r="B4" s="10">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>182</v>
+        <v>162</v>
       </c>
       <c r="E4" s="1">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>279</v>
       </c>
       <c r="G4" s="1">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H4" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F4,"&lt;",G4,"&gt;"" LOC = ",$C4," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;2&gt;" LOC = P12 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;7&gt;" LOC = P27 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I4" s="1">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J4" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F4,"&lt;",I4,"&gt;"" LOC = ",$C4," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;2&gt;" LOC = P12 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;7&gt;" LOC = P27 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K4" s="1">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L4" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>NET "A&lt;2&gt;" LOC = P12 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F4,"&lt;",K4,"&gt;"" LOC = ",$C4," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;7&gt;" LOC = P27 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -4498,40 +4498,40 @@
         <v>238</v>
       </c>
       <c r="B5" s="10">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="E5" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>279</v>
       </c>
       <c r="G5" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H5" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F5,"&lt;",G5,"&gt;"" LOC = ",$C5," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;3&gt;" LOC = P15 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;6&gt;" LOC = P24 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I5" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J5" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F5,"&lt;",I5,"&gt;"" LOC = ",$C5," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;3&gt;" LOC = P15 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;6&gt;" LOC = P24 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K5" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L5" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>NET "A&lt;3&gt;" LOC = P15 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F5,"&lt;",K5,"&gt;"" LOC = ",$C5," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;6&gt;" LOC = P24 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -4539,40 +4539,40 @@
         <v>238</v>
       </c>
       <c r="B6" s="10">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="E6" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>279</v>
       </c>
       <c r="G6" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H6" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F6,"&lt;",G6,"&gt;"" LOC = ",$C6," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;4&gt;" LOC = P17 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;5&gt;" LOC = P22 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I6" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J6" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F6,"&lt;",I6,"&gt;"" LOC = ",$C6," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;4&gt;" LOC = P17 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;5&gt;" LOC = P22 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K6" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L6" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>NET "A&lt;4&gt;" LOC = P17 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F6,"&lt;",K6,"&gt;"" LOC = ",$C6," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;5&gt;" LOC = P22 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -4580,40 +4580,40 @@
         <v>238</v>
       </c>
       <c r="B7" s="10">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="E7" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>279</v>
       </c>
       <c r="G7" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H7" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F7,"&lt;",G7,"&gt;"" LOC = ",$C7," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;5&gt;" LOC = P22 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;4&gt;" LOC = P17 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I7" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J7" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F7,"&lt;",I7,"&gt;"" LOC = ",$C7," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;5&gt;" LOC = P22 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;4&gt;" LOC = P17 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K7" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L7" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>NET "A&lt;5&gt;" LOC = P22 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F7,"&lt;",K7,"&gt;"" LOC = ",$C7," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;4&gt;" LOC = P17 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -4621,40 +4621,40 @@
         <v>238</v>
       </c>
       <c r="B8" s="10">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="E8" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>279</v>
       </c>
       <c r="G8" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H8" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F8,"&lt;",G8,"&gt;"" LOC = ",$C8," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;6&gt;" LOC = P24 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;3&gt;" LOC = P15 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I8" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J8" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F8,"&lt;",I8,"&gt;"" LOC = ",$C8," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;6&gt;" LOC = P24 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;3&gt;" LOC = P15 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K8" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L8" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>NET "A&lt;6&gt;" LOC = P24 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F8,"&lt;",K8,"&gt;"" LOC = ",$C8," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;3&gt;" LOC = P15 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -4662,40 +4662,40 @@
         <v>238</v>
       </c>
       <c r="B9" s="10">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>161</v>
+        <v>181</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>162</v>
+        <v>182</v>
       </c>
       <c r="E9" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>279</v>
       </c>
       <c r="G9" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H9" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F9,"&lt;",G9,"&gt;"" LOC = ",$C9," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;7&gt;" LOC = P27 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;2&gt;" LOC = P12 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I9" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J9" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F9,"&lt;",I9,"&gt;"" LOC = ",$C9," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;7&gt;" LOC = P27 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;2&gt;" LOC = P12 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K9" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L9" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>NET "A&lt;7&gt;" LOC = P27 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F9,"&lt;",K9,"&gt;"" LOC = ",$C9," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;2&gt;" LOC = P12 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -4703,40 +4703,40 @@
         <v>238</v>
       </c>
       <c r="B10" s="10">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="E10" s="1">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>279</v>
       </c>
       <c r="G10" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H10" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F10,"&lt;",G10,"&gt;"" LOC = ",$C10," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;8&gt;" LOC = P23 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;1&gt;" LOC = P10 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I10" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J10" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F10,"&lt;",I10,"&gt;"" LOC = ",$C10," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;8&gt;" LOC = P23 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;1&gt;" LOC = P10 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K10" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L10" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>NET "A&lt;8&gt;" LOC = P23 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F10,"&lt;",K10,"&gt;"" LOC = ",$C10," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;1&gt;" LOC = P10 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -4744,40 +4744,40 @@
         <v>238</v>
       </c>
       <c r="B11" s="10">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>171</v>
+        <v>189</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="E11" s="1">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>279</v>
       </c>
       <c r="G11" s="1">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H11" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F11,"&lt;",G11,"&gt;"" LOC = ",$C11," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;9&gt;" LOC = P21 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;0&gt;" LOC = P8 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I11" s="1">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J11" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F11,"&lt;",I11,"&gt;"" LOC = ",$C11," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;9&gt;" LOC = P21 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;0&gt;" LOC = P8 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K11" s="1">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L11" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>NET "A&lt;9&gt;" LOC = P21 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F11,"&lt;",K11,"&gt;"" LOC = ",$C11," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;0&gt;" LOC = P8 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -4785,40 +4785,40 @@
         <v>238</v>
       </c>
       <c r="B12" s="10">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="E12" s="1">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>279</v>
+        <v>295</v>
       </c>
       <c r="G12" s="1">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H12" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F12,"&lt;",G12,"&gt;"" LOC = ",$C12," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;10&gt;" LOC = P11 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;0&gt;" LOC = P6 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I12" s="1">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J12" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F12,"&lt;",I12,"&gt;"" LOC = ",$C12," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;10&gt;" LOC = P11 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;0&gt;" LOC = P6 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K12" s="1">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L12" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>NET "A&lt;10&gt;" LOC = P11 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F12,"&lt;",K12,"&gt;"" LOC = ",$C12," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "D&lt;0&gt;" LOC = P6 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -4826,40 +4826,40 @@
         <v>238</v>
       </c>
       <c r="B13" s="10">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>175</v>
+        <v>197</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>176</v>
+        <v>198</v>
       </c>
       <c r="E13" s="1">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>279</v>
+        <v>295</v>
       </c>
       <c r="G13" s="1">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="H13" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F13,"&lt;",G13,"&gt;"" LOC = ",$C13," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;11&gt;" LOC = P16 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;1&gt;" LOC = P2 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I13" s="1">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="J13" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F13,"&lt;",I13,"&gt;"" LOC = ",$C13," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;11&gt;" LOC = P16 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;1&gt;" LOC = P2 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K13" s="1">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="L13" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>NET "A&lt;11&gt;" LOC = P16 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F13,"&lt;",K13,"&gt;"" LOC = ",$C13," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "D&lt;1&gt;" LOC = P2 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -4867,40 +4867,40 @@
         <v>238</v>
       </c>
       <c r="B14" s="10">
+        <v>35</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="E14" s="1">
         <v>13</v>
       </c>
-      <c r="C14" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="D14" s="20" t="s">
-        <v>158</v>
-      </c>
-      <c r="E14" s="1">
+      <c r="F14" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="G14" s="1">
         <v>2</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="G14" s="1">
-        <v>12</v>
       </c>
       <c r="H14" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F14,"&lt;",G14,"&gt;"" LOC = ",$C14," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;12&gt;" LOC = P30 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;2&gt;" LOC = P144 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I14" s="1">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J14" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F14,"&lt;",I14,"&gt;"" LOC = ",$C14," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;12&gt;" LOC = P30 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;2&gt;" LOC = P144 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K14" s="1">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="L14" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>NET "A&lt;12&gt;" LOC = P30 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F14,"&lt;",K14,"&gt;"" LOC = ",$C14," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "D&lt;2&gt;" LOC = P144 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -4908,40 +4908,40 @@
         <v>238</v>
       </c>
       <c r="B15" s="10">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>163</v>
+        <v>6</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>164</v>
+        <v>7</v>
       </c>
       <c r="E15" s="1">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>279</v>
+        <v>295</v>
       </c>
       <c r="G15" s="1">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="H15" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F15,"&lt;",G15,"&gt;"" LOC = ",$C15," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;13&gt;" LOC = P26 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;3&gt;" LOC = P141 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I15" s="1">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="J15" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F15,"&lt;",I15,"&gt;"" LOC = ",$C15," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;13&gt;" LOC = P26 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;3&gt;" LOC = P141 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K15" s="1">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="L15" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>NET "A&lt;13&gt;" LOC = P26 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F15,"&lt;",K15,"&gt;"" LOC = ",$C15," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "D&lt;3&gt;" LOC = P141 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -4949,40 +4949,40 @@
         <v>238</v>
       </c>
       <c r="B16" s="10">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>159</v>
+        <v>2</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>160</v>
-      </c>
-      <c r="E16" s="13">
-        <v>27</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>279</v>
-      </c>
-      <c r="G16" s="13">
-        <v>14</v>
-      </c>
-      <c r="H16" s="13" t="str">
+        <v>3</v>
+      </c>
+      <c r="E16" s="1">
+        <v>16</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="G16" s="1">
+        <v>4</v>
+      </c>
+      <c r="H16" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F16,"&lt;",G16,"&gt;"" LOC = ",$C16," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;14&gt;" LOC = P29 | IOSTANDARD = LVCMOS33;</v>
-      </c>
-      <c r="I16" s="13">
-        <v>14</v>
+        <v>NET "D&lt;4&gt;" LOC = P143 | IOSTANDARD = LVCMOS33;</v>
+      </c>
+      <c r="I16" s="1">
+        <v>4</v>
       </c>
       <c r="J16" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F16,"&lt;",I16,"&gt;"" LOC = ",$C16," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;14&gt;" LOC = P29 | IOSTANDARD = LVCMOS33;</v>
-      </c>
-      <c r="K16" s="13" t="s">
-        <v>296</v>
-      </c>
-      <c r="L16" s="13" t="str">
-        <f xml:space="preserve"> CONCATENATE("NET """,K16,""" LOC = ",$C16," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "WE" LOC = P29 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;4&gt;" LOC = P143 | IOSTANDARD = LVCMOS33;</v>
+      </c>
+      <c r="K16" s="1">
+        <v>4</v>
+      </c>
+      <c r="L16" s="1" t="str">
+        <f xml:space="preserve"> CONCATENATE("NET """,$F16,"&lt;",K16,"&gt;"" LOC = ",$C16," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "D&lt;4&gt;" LOC = P143 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
@@ -4990,40 +4990,40 @@
         <v>238</v>
       </c>
       <c r="B17" s="10">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>153</v>
+        <v>199</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="E17" s="13">
-        <v>1</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>279</v>
-      </c>
-      <c r="G17" s="13">
-        <v>15</v>
-      </c>
-      <c r="H17" s="13" t="str">
+        <v>200</v>
+      </c>
+      <c r="E17" s="1">
+        <v>17</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="G17" s="1">
+        <v>5</v>
+      </c>
+      <c r="H17" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F17,"&lt;",G17,"&gt;"" LOC = ",$C17," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;15&gt;" LOC = P33 | IOSTANDARD = LVCMOS33;</v>
-      </c>
-      <c r="I17" s="13" t="s">
-        <v>300</v>
-      </c>
-      <c r="J17" s="13" t="str">
-        <f xml:space="preserve"> CONCATENATE("NET """,I17,""" LOC = ",$C17," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "VPP" LOC = P33 | IOSTANDARD = LVCMOS33;</v>
-      </c>
-      <c r="K17" s="13">
-        <v>14</v>
-      </c>
-      <c r="L17" s="13" t="str">
+        <v>NET "D&lt;5&gt;" LOC = P1 | IOSTANDARD = LVCMOS33;</v>
+      </c>
+      <c r="I17" s="1">
+        <v>5</v>
+      </c>
+      <c r="J17" s="1" t="str">
+        <f xml:space="preserve"> CONCATENATE("NET """,$F17,"&lt;",I17,"&gt;"" LOC = ",$C17," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "D&lt;5&gt;" LOC = P1 | IOSTANDARD = LVCMOS33;</v>
+      </c>
+      <c r="K17" s="1">
+        <v>5</v>
+      </c>
+      <c r="L17" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F17,"&lt;",K17,"&gt;"" LOC = ",$C17," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "A&lt;14&gt;" LOC = P33 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;5&gt;" LOC = P1 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
@@ -5031,40 +5031,40 @@
         <v>238</v>
       </c>
       <c r="B18" s="10">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E18" s="1">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>295</v>
       </c>
       <c r="G18" s="1">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H18" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F18,"&lt;",G18,"&gt;"" LOC = ",$C18," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;0&gt;" LOC = P6 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;6&gt;" LOC = P5 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I18" s="1">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J18" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F18,"&lt;",I18,"&gt;"" LOC = ",$C18," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;0&gt;" LOC = P6 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;6&gt;" LOC = P5 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K18" s="1">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L18" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F18,"&lt;",K18,"&gt;"" LOC = ",$C18," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;0&gt;" LOC = P6 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;6&gt;" LOC = P5 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
@@ -5072,40 +5072,40 @@
         <v>238</v>
       </c>
       <c r="B19" s="10">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="E19" s="1">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>295</v>
       </c>
       <c r="G19" s="1">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H19" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F19,"&lt;",G19,"&gt;"" LOC = ",$C19," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;1&gt;" LOC = P2 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;7&gt;" LOC = P7 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I19" s="1">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J19" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F19,"&lt;",I19,"&gt;"" LOC = ",$C19," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;1&gt;" LOC = P2 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "D&lt;7&gt;" LOC = P7 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K19" s="1">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L19" s="1" t="str">
-        <f t="shared" ref="L19:L25" si="1" xml:space="preserve"> CONCATENATE("NET """,$F19,"&lt;",K19,"&gt;"" LOC = ",$C19," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;1&gt;" LOC = P2 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F19,"&lt;",K19,"&gt;"" LOC = ",$C19," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "D&lt;7&gt;" LOC = P7 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
@@ -5113,40 +5113,38 @@
         <v>238</v>
       </c>
       <c r="B20" s="10">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>0</v>
+        <v>187</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="E20" s="1">
-        <v>13</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>295</v>
-      </c>
-      <c r="G20" s="1">
-        <v>2</v>
-      </c>
-      <c r="H20" s="1" t="str">
-        <f xml:space="preserve"> CONCATENATE("NET """,$F20,"&lt;",G20,"&gt;"" LOC = ",$C20," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;2&gt;" LOC = P144 | IOSTANDARD = LVCMOS33;</v>
-      </c>
-      <c r="I20" s="1">
-        <v>2</v>
-      </c>
-      <c r="J20" s="1" t="str">
-        <f xml:space="preserve"> CONCATENATE("NET """,$F20,"&lt;",I20,"&gt;"" LOC = ",$C20," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;2&gt;" LOC = P144 | IOSTANDARD = LVCMOS33;</v>
-      </c>
-      <c r="K20" s="1">
-        <v>2</v>
-      </c>
-      <c r="L20" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>NET "D&lt;2&gt;" LOC = P144 | IOSTANDARD = LVCMOS33;</v>
+        <v>188</v>
+      </c>
+      <c r="E20" s="13">
+        <v>20</v>
+      </c>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="H20" s="13" t="str">
+        <f xml:space="preserve"> CONCATENATE("NET """,$G20,""" LOC = ",$C20," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "CE" LOC = P9 | IOSTANDARD = LVCMOS33;</v>
+      </c>
+      <c r="I20" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="J20" s="13" t="str">
+        <f xml:space="preserve"> CONCATENATE("NET """,$I20,""" LOC = ",$C20," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "CE" LOC = P9 | IOSTANDARD = LVCMOS33;</v>
+      </c>
+      <c r="K20" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="L20" s="13" t="str">
+        <f xml:space="preserve"> CONCATENATE("NET """,K20,""" LOC = ",$C20," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "CE" LOC = P9 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
@@ -5154,40 +5152,40 @@
         <v>238</v>
       </c>
       <c r="B21" s="10">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>6</v>
+        <v>183</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>7</v>
+        <v>184</v>
       </c>
       <c r="E21" s="1">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>295</v>
+        <v>279</v>
       </c>
       <c r="G21" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H21" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F21,"&lt;",G21,"&gt;"" LOC = ",$C21," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;3&gt;" LOC = P141 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;10&gt;" LOC = P11 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I21" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J21" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F21,"&lt;",I21,"&gt;"" LOC = ",$C21," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;3&gt;" LOC = P141 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;10&gt;" LOC = P11 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K21" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L21" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>NET "D&lt;3&gt;" LOC = P141 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F21,"&lt;",K21,"&gt;"" LOC = ",$C21," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;10&gt;" LOC = P11 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
@@ -5195,40 +5193,38 @@
         <v>238</v>
       </c>
       <c r="B22" s="10">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>2</v>
+        <v>179</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="E22" s="1">
-        <v>16</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>295</v>
-      </c>
-      <c r="G22" s="1">
-        <v>4</v>
-      </c>
-      <c r="H22" s="1" t="str">
-        <f xml:space="preserve"> CONCATENATE("NET """,$F22,"&lt;",G22,"&gt;"" LOC = ",$C22," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;4&gt;" LOC = P143 | IOSTANDARD = LVCMOS33;</v>
-      </c>
-      <c r="I22" s="1">
-        <v>4</v>
-      </c>
-      <c r="J22" s="1" t="str">
-        <f xml:space="preserve"> CONCATENATE("NET """,$F22,"&lt;",I22,"&gt;"" LOC = ",$C22," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;4&gt;" LOC = P143 | IOSTANDARD = LVCMOS33;</v>
-      </c>
-      <c r="K22" s="1">
-        <v>4</v>
-      </c>
-      <c r="L22" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>NET "D&lt;4&gt;" LOC = P143 | IOSTANDARD = LVCMOS33;</v>
+        <v>180</v>
+      </c>
+      <c r="E22" s="13">
+        <v>22</v>
+      </c>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="H22" s="13" t="str">
+        <f xml:space="preserve"> CONCATENATE("NET """,$G22,""" LOC = ",$C22," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "OE" LOC = P14 | IOSTANDARD = LVCMOS33;</v>
+      </c>
+      <c r="I22" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="J22" s="13" t="str">
+        <f xml:space="preserve"> CONCATENATE("NET """,$I22,""" LOC = ",$C22," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "OE" LOC = P14 | IOSTANDARD = LVCMOS33;</v>
+      </c>
+      <c r="K22" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="L22" s="13" t="str">
+        <f xml:space="preserve"> CONCATENATE("NET """,K22,""" LOC = ",$C22," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "OE" LOC = P14 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
@@ -5236,40 +5232,40 @@
         <v>238</v>
       </c>
       <c r="B23" s="10">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>199</v>
+        <v>175</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>200</v>
+        <v>176</v>
       </c>
       <c r="E23" s="1">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>295</v>
+        <v>279</v>
       </c>
       <c r="G23" s="1">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H23" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F23,"&lt;",G23,"&gt;"" LOC = ",$C23," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;5&gt;" LOC = P1 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;11&gt;" LOC = P16 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I23" s="1">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="J23" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F23,"&lt;",I23,"&gt;"" LOC = ",$C23," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;5&gt;" LOC = P1 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;11&gt;" LOC = P16 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K23" s="1">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="L23" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>NET "D&lt;5&gt;" LOC = P1 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F23,"&lt;",K23,"&gt;"" LOC = ",$C23," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;11&gt;" LOC = P16 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
@@ -5277,40 +5273,40 @@
         <v>238</v>
       </c>
       <c r="B24" s="10">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>195</v>
+        <v>171</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>196</v>
+        <v>172</v>
       </c>
       <c r="E24" s="1">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>295</v>
+        <v>279</v>
       </c>
       <c r="G24" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H24" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F24,"&lt;",G24,"&gt;"" LOC = ",$C24," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;6&gt;" LOC = P5 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;9&gt;" LOC = P21 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I24" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J24" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F24,"&lt;",I24,"&gt;"" LOC = ",$C24," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;6&gt;" LOC = P5 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;9&gt;" LOC = P21 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K24" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L24" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>NET "D&lt;6&gt;" LOC = P5 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F24,"&lt;",K24,"&gt;"" LOC = ",$C24," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;9&gt;" LOC = P21 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
@@ -5318,40 +5314,40 @@
         <v>238</v>
       </c>
       <c r="B25" s="10">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>191</v>
+        <v>167</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>192</v>
+        <v>168</v>
       </c>
       <c r="E25" s="1">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>295</v>
+        <v>279</v>
       </c>
       <c r="G25" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H25" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F25,"&lt;",G25,"&gt;"" LOC = ",$C25," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;7&gt;" LOC = P7 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;8&gt;" LOC = P23 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="I25" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J25" s="1" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,$F25,"&lt;",I25,"&gt;"" LOC = ",$C25," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "D&lt;7&gt;" LOC = P7 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "A&lt;8&gt;" LOC = P23 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K25" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L25" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>NET "D&lt;7&gt;" LOC = P7 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F25,"&lt;",K25,"&gt;"" LOC = ",$C25," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;8&gt;" LOC = P23 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
@@ -5359,38 +5355,40 @@
         <v>238</v>
       </c>
       <c r="B26" s="10">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>187</v>
+        <v>163</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>188</v>
-      </c>
-      <c r="E26" s="13">
-        <v>20</v>
-      </c>
-      <c r="F26" s="13"/>
-      <c r="G26" s="13" t="s">
-        <v>292</v>
-      </c>
-      <c r="H26" s="13" t="str">
-        <f xml:space="preserve"> CONCATENATE("NET """,$G26,""" LOC = ",$C26," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "CE" LOC = P9 | IOSTANDARD = LVCMOS33;</v>
-      </c>
-      <c r="I26" s="13" t="s">
-        <v>292</v>
-      </c>
-      <c r="J26" s="13" t="str">
-        <f xml:space="preserve"> CONCATENATE("NET """,$I26,""" LOC = ",$C26," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "CE" LOC = P9 | IOSTANDARD = LVCMOS33;</v>
-      </c>
-      <c r="K26" s="13" t="s">
-        <v>292</v>
-      </c>
-      <c r="L26" s="13" t="str">
-        <f xml:space="preserve"> CONCATENATE("NET """,K26,""" LOC = ",$C26," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "CE" LOC = P9 | IOSTANDARD = LVCMOS33;</v>
+        <v>164</v>
+      </c>
+      <c r="E26" s="1">
+        <v>26</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="G26" s="1">
+        <v>13</v>
+      </c>
+      <c r="H26" s="1" t="str">
+        <f xml:space="preserve"> CONCATENATE("NET """,$F26,"&lt;",G26,"&gt;"" LOC = ",$C26," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;13&gt;" LOC = P26 | IOSTANDARD = LVCMOS33;</v>
+      </c>
+      <c r="I26" s="1">
+        <v>13</v>
+      </c>
+      <c r="J26" s="1" t="str">
+        <f xml:space="preserve"> CONCATENATE("NET """,$F26,"&lt;",I26,"&gt;"" LOC = ",$C26," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;13&gt;" LOC = P26 | IOSTANDARD = LVCMOS33;</v>
+      </c>
+      <c r="K26" s="1">
+        <v>13</v>
+      </c>
+      <c r="L26" s="1" t="str">
+        <f xml:space="preserve"> CONCATENATE("NET """,$F26,"&lt;",K26,"&gt;"" LOC = ",$C26," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;13&gt;" LOC = P26 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
@@ -5398,38 +5396,40 @@
         <v>238</v>
       </c>
       <c r="B27" s="10">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>179</v>
+        <v>159</v>
       </c>
       <c r="D27" s="20" t="s">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="E27" s="13">
-        <v>22</v>
-      </c>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13" t="s">
-        <v>293</v>
+        <v>27</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>279</v>
+      </c>
+      <c r="G27" s="13">
+        <v>14</v>
       </c>
       <c r="H27" s="13" t="str">
-        <f xml:space="preserve"> CONCATENATE("NET """,$G27,""" LOC = ",$C27," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "OE" LOC = P14 | IOSTANDARD = LVCMOS33;</v>
-      </c>
-      <c r="I27" s="13" t="s">
-        <v>293</v>
-      </c>
-      <c r="J27" s="13" t="str">
-        <f xml:space="preserve"> CONCATENATE("NET """,$I27,""" LOC = ",$C27," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "OE" LOC = P14 | IOSTANDARD = LVCMOS33;</v>
+        <f xml:space="preserve"> CONCATENATE("NET """,$F27,"&lt;",G27,"&gt;"" LOC = ",$C27," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;14&gt;" LOC = P29 | IOSTANDARD = LVCMOS33;</v>
+      </c>
+      <c r="I27" s="13">
+        <v>14</v>
+      </c>
+      <c r="J27" s="1" t="str">
+        <f xml:space="preserve"> CONCATENATE("NET """,$F27,"&lt;",I27,"&gt;"" LOC = ",$C27," | IOSTANDARD = LVCMOS33;")</f>
+        <v>NET "A&lt;14&gt;" LOC = P29 | IOSTANDARD = LVCMOS33;</v>
       </c>
       <c r="K27" s="13" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="L27" s="13" t="str">
         <f xml:space="preserve"> CONCATENATE("NET """,K27,""" LOC = ",$C27," | IOSTANDARD = LVCMOS33;")</f>
-        <v>NET "OE" LOC = P14 | IOSTANDARD = LVCMOS33;</v>
+        <v>NET "WE" LOC = P29 | IOSTANDARD = LVCMOS33;</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
@@ -5451,8 +5451,8 @@
       <c r="L33" s="1"/>
     </row>
   </sheetData>
-  <sortState ref="A2:G31">
-    <sortCondition ref="G2:G31"/>
+  <sortState ref="A2:L33">
+    <sortCondition ref="E2:E33"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>